<commit_message>
add: shleeclay 게재논문 — Bi-temporal ALS forest structures (Forest Science and Technology, 2026, SCI Q2) 게재 반영
- Under Review에서 제거(→4편), Publications id10 추가(웹 카드·CV)
- citation bib(lee2026_fst) 추가·병합, citations.json 재생성
- CV v11 승격·배포 PDF 교체, v10→old/, 기준선 갱신
- 표지 이미지·PDF·figure는 추후 제공 예정
</commit_message>
<xml_diff>
--- a/cv/citations/publications.xlsx
+++ b/cv/citations/publications.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'publications'!$A$1:$K$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'publications'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -976,8 +976,49 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Forest Science and Technology</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Bi-temporal ALS assessment of vertical–horizontal forest structures and their structural association in a temperate urban forest</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Lee, Seunghyeon and Kim, Yonghwan and Kim, Dohee and Kim, Hansoo and Song, Youngkeun</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>10.1080/21580103.2026.2712965</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K10"/>
+  <autoFilter ref="A1:K11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -988,6 +1029,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>